<commit_message>
Task 3 — Event Impact ModelingModeling how events (policies, product launches, infrastructure investments)affect financial inclusion indicators, using the `impact_links` records from the enriched dataset.
</commit_message>
<xml_diff>
--- a/data/processed/ethiopia_fi_unified_data_enriched.xlsx
+++ b/data/processed/ethiopia_fi_unified_data_enriched.xlsx
@@ -5241,10 +5241,8 @@
           <t>agents</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>2022-09-30</t>
-        </is>
+      <c r="L45" s="1" t="n">
+        <v>44834</v>
       </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
@@ -5357,10 +5355,8 @@
           <t>agents</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>2023-07-01</t>
-        </is>
+      <c r="L46" s="1" t="n">
+        <v>45108</v>
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
@@ -5473,10 +5469,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>2023-06-30</t>
-        </is>
+      <c r="L47" s="1" t="n">
+        <v>45107</v>
       </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
@@ -5589,10 +5583,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>2023-06-30</t>
-        </is>
+      <c r="L48" s="1" t="n">
+        <v>45107</v>
       </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
@@ -5705,10 +5697,8 @@
           <t>loans</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>2023-07-01</t>
-        </is>
+      <c r="L49" s="1" t="n">
+        <v>45108</v>
       </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
@@ -5821,10 +5811,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>2023-01-15</t>
-        </is>
+      <c r="L50" s="1" t="n">
+        <v>44941</v>
       </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
@@ -5937,10 +5925,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>2024-01-15</t>
-        </is>
+      <c r="L51" s="1" t="n">
+        <v>45306</v>
       </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
@@ -6053,10 +6039,8 @@
           <t>%</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
+      <c r="L52" s="1" t="n">
+        <v>46215</v>
       </c>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
@@ -6151,10 +6135,8 @@
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>2023-10-09</t>
-        </is>
+      <c r="L53" s="1" t="n">
+        <v>45208</v>
       </c>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
@@ -6241,10 +6223,8 @@
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>2025-05-27</t>
-        </is>
+      <c r="L54" s="1" t="n">
+        <v>45804</v>
       </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
@@ -6331,10 +6311,8 @@
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>2023-09-01</t>
-        </is>
+      <c r="L55" s="1" t="n">
+        <v>45170</v>
       </c>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
@@ -6421,10 +6399,8 @@
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>2026-07-12</t>
-        </is>
+      <c r="L56" s="1" t="n">
+        <v>46215</v>
       </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>

</xml_diff>